<commit_message>
Generate Blue Crew pairings schedule; update to 9-round format
- docs/BlueCrew_Pairings.xlsx: full pairings schedule for Blue Crew (JPL Team)
  generated by new backend/generate_pairings.py script
  Trevor/Alexis draw 3 mixed games; Arman/Richard play 4 games (both unavoidable)
  couples always play together in mixed; no man repeats a partner
- src/data/mockData.js: real player names for both teams (Hill Street Blues + Blue Crew)
  corrected to 9 rounds / 18 matches matching actual tournament docx
- backend/code.gs: initSheets updated to 18 match slots (m1–m18, 9 rounds)
- backend/generate_template.py: real Blue Crew names; corrected to 9-round schedule
- backend/ATH_Open_Sheets_Template.xlsx: regenerated with real names + 9 rounds
- ATHOPEN.md: all sections updated to reflect 9-round format and completed pairings

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/ATH_Open_Sheets_Template.xlsx
+++ b/backend/ATH_Open_Sheets_Template.xlsx
@@ -1196,14 +1196,10 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Cora</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Williams</t>
-        </is>
-      </c>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
       <c r="D15" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1220,20 +1216,12 @@
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr"/>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0001</t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>cora@example.com</t>
-        </is>
-      </c>
+      <c r="H15" s="4" t="inlineStr"/>
+      <c r="I15" s="4" t="inlineStr"/>
       <c r="J15" s="4" t="inlineStr"/>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>b8</t>
+          <t>b6</t>
         </is>
       </c>
     </row>
@@ -1245,14 +1233,10 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Sofia</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Reyes</t>
-        </is>
-      </c>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr"/>
       <c r="D16" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1269,20 +1253,12 @@
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr"/>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0009</t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>sofia@example.com</t>
-        </is>
-      </c>
+      <c r="H16" s="4" t="inlineStr"/>
+      <c r="I16" s="4" t="inlineStr"/>
       <c r="J16" s="4" t="inlineStr"/>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>b11</t>
+          <t>b3</t>
         </is>
       </c>
     </row>
@@ -1294,14 +1270,10 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Maria</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Kim</t>
-        </is>
-      </c>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr"/>
       <c r="D17" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1318,16 +1290,8 @@
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0010</t>
-        </is>
-      </c>
-      <c r="I17" s="4" t="inlineStr">
-        <is>
-          <t>maria@example.com</t>
-        </is>
-      </c>
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr"/>
       <c r="J17" s="4" t="inlineStr"/>
       <c r="K17" s="4" t="inlineStr">
         <is>
@@ -1343,14 +1307,10 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Paul</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>Jensen</t>
-        </is>
-      </c>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr"/>
       <c r="D18" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1367,16 +1327,8 @@
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0002</t>
-        </is>
-      </c>
-      <c r="I18" s="4" t="inlineStr">
-        <is>
-          <t>paul@example.com</t>
-        </is>
-      </c>
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr"/>
       <c r="J18" s="4" t="inlineStr"/>
       <c r="K18" s="4" t="inlineStr"/>
     </row>
@@ -1388,14 +1340,10 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Raj</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Patel</t>
-        </is>
-      </c>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr"/>
       <c r="D19" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1412,18 +1360,14 @@
         </is>
       </c>
       <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0003</t>
-        </is>
-      </c>
-      <c r="I19" s="4" t="inlineStr">
-        <is>
-          <t>raj@example.com</t>
-        </is>
-      </c>
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr"/>
       <c r="J19" s="4" t="inlineStr"/>
-      <c r="K19" s="4" t="inlineStr"/>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>b9</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1433,14 +1377,10 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Tom</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Nguyen</t>
-        </is>
-      </c>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr"/>
       <c r="D20" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1457,16 +1397,8 @@
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0004</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>tom@example.com</t>
-        </is>
-      </c>
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr"/>
       <c r="J20" s="4" t="inlineStr"/>
       <c r="K20" s="4" t="inlineStr"/>
     </row>
@@ -1478,14 +1410,10 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Eric</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>Hall</t>
-        </is>
-      </c>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1502,16 +1430,8 @@
         </is>
       </c>
       <c r="G21" s="4" t="inlineStr"/>
-      <c r="H21" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0005</t>
-        </is>
-      </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>eric@example.com</t>
-        </is>
-      </c>
+      <c r="H21" s="4" t="inlineStr"/>
+      <c r="I21" s="4" t="inlineStr"/>
       <c r="J21" s="4" t="inlineStr"/>
       <c r="K21" s="4" t="inlineStr"/>
     </row>
@@ -1523,14 +1443,10 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Diego</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Castro</t>
-        </is>
-      </c>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr"/>
       <c r="D22" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1547,18 +1463,14 @@
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr"/>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0006</t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>diego@example.com</t>
-        </is>
-      </c>
+      <c r="H22" s="4" t="inlineStr"/>
+      <c r="I22" s="4" t="inlineStr"/>
       <c r="J22" s="4" t="inlineStr"/>
-      <c r="K22" s="4" t="inlineStr"/>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>b1</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1568,14 +1480,10 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Nathan</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Ford</t>
-        </is>
-      </c>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr"/>
       <c r="D23" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1592,16 +1500,8 @@
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr"/>
-      <c r="H23" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0007</t>
-        </is>
-      </c>
-      <c r="I23" s="4" t="inlineStr">
-        <is>
-          <t>nathan@example.com</t>
-        </is>
-      </c>
+      <c r="H23" s="4" t="inlineStr"/>
+      <c r="I23" s="4" t="inlineStr"/>
       <c r="J23" s="4" t="inlineStr"/>
       <c r="K23" s="4" t="inlineStr"/>
     </row>
@@ -1613,14 +1513,10 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Omar</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Diallo</t>
-        </is>
-      </c>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1637,22 +1533,10 @@
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr"/>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0008</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>omar@example.com</t>
-        </is>
-      </c>
+      <c r="H24" s="4" t="inlineStr"/>
+      <c r="I24" s="4" t="inlineStr"/>
       <c r="J24" s="4" t="inlineStr"/>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>b1</t>
-        </is>
-      </c>
+      <c r="K24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1662,14 +1546,10 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Carlos</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Reyes</t>
-        </is>
-      </c>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr"/>
       <c r="D25" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1686,22 +1566,10 @@
         </is>
       </c>
       <c r="G25" s="4" t="inlineStr"/>
-      <c r="H25" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0011</t>
-        </is>
-      </c>
-      <c r="I25" s="4" t="inlineStr">
-        <is>
-          <t>carlos@example.com</t>
-        </is>
-      </c>
+      <c r="H25" s="4" t="inlineStr"/>
+      <c r="I25" s="4" t="inlineStr"/>
       <c r="J25" s="4" t="inlineStr"/>
-      <c r="K25" s="4" t="inlineStr">
-        <is>
-          <t>b9</t>
-        </is>
-      </c>
+      <c r="K25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1711,14 +1579,10 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>James</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>Kim</t>
-        </is>
-      </c>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr"/>
       <c r="D26" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -1735,16 +1599,8 @@
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr"/>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t>(555)200-0012</t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>james@example.com</t>
-        </is>
-      </c>
+      <c r="H26" s="4" t="inlineStr"/>
+      <c r="I26" s="4" t="inlineStr"/>
       <c r="J26" s="4" t="inlineStr"/>
       <c r="K26" s="4" t="inlineStr">
         <is>
@@ -1763,7 +1619,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1925,54 +1781,54 @@
       <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>m5</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
-      <c r="G6" s="6" t="inlineStr"/>
-      <c r="H6" s="6" t="inlineStr"/>
-      <c r="I6" s="6" t="inlineStr"/>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr"/>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>m6</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>TRUE</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
-      <c r="G7" s="6" t="inlineStr"/>
-      <c r="H7" s="6" t="inlineStr"/>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -2000,54 +1856,54 @@
       <c r="I8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>m8</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
-      <c r="G9" s="5" t="inlineStr"/>
-      <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr"/>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>m9</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="inlineStr"/>
-      <c r="F10" s="5" t="inlineStr"/>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
-      <c r="I10" s="5" t="inlineStr"/>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="6" t="inlineStr"/>
+      <c r="G10" s="6" t="inlineStr"/>
+      <c r="H10" s="6" t="inlineStr"/>
+      <c r="I10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -2075,104 +1931,104 @@
       <c r="I11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>m11</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="H12" s="5" t="inlineStr"/>
+      <c r="I12" s="5" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>m12</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr"/>
+      <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="5" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>m13</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="6" t="inlineStr"/>
-      <c r="G12" s="6" t="inlineStr"/>
-      <c r="H12" s="6" t="inlineStr"/>
-      <c r="I12" s="6" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>m12</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="6" t="inlineStr"/>
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr"/>
+      <c r="I14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>m14</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D13" s="6" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="6" t="inlineStr"/>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="6" t="inlineStr"/>
-      <c r="I13" s="6" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>m13</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>S</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="inlineStr"/>
-      <c r="F14" s="5" t="inlineStr"/>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr"/>
-      <c r="I14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>m14</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
-      <c r="G15" s="5" t="inlineStr"/>
-      <c r="H15" s="5" t="inlineStr"/>
-      <c r="I15" s="5" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -2223,6 +2079,56 @@
       <c r="G17" s="5" t="inlineStr"/>
       <c r="H17" s="5" t="inlineStr"/>
       <c r="I17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>m17</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="6" t="inlineStr"/>
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr"/>
+      <c r="I18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>m18</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>TRUE</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="6" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr"/>
+      <c r="H19" s="6" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2238,7 +2144,7 @@
   <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2412,7 +2318,7 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>TRUE = Mixed Doubles ★  (yellow rows). Pre-filled.</t>
+          <t>TRUE = Mixed Doubles ★ (yellow rows). Pre-filled.</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2330,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>Team A player IDs for this match (copy from Players tab column A)</t>
+          <t>Team A player IDs for this match — copy from Players tab column A</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2377,7 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>Players with a partnerId play together in all Mixed Doubles matches (★ rows).</t>
+          <t>Players with a partnerId play together in all Mixed Doubles (★) matches.</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2389,7 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>Captain plays 1 mixed doubles game (round 4 South). Her partner plays 1 mixed + 2 men's.</t>
+          <t>Captain plays 1 mixed game (round 4 South). Her partner: 1 mixed + 2 men's.</t>
         </is>
       </c>
     </row>
@@ -2495,7 +2401,7 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>Each plays 2 mixed doubles games (rounds 3 and 6). Their partners play 2 mixed + 1 men's.</t>
+          <t>Each plays 2 mixed games (rounds 3 and 6). Their partners: 2 mixed + 1 men's.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Full Schedule, HSB/Blue Crew pairings matrix and player summary sheets to template
generate_template.py now produces 8 sheets:
- Players, Schedule, How To Use (existing)
- Full Schedule: all 18 matches with both teams' player names
- HSB Pairings Matrix: 12×12 player grid (X=men's, M★=mixed, color-coded)
- HSB Player Summary: per-player game counts + partners in order
- Blue Crew Matrix: 13×13 grid with C★ captain's game, orange for 4-game players
- Blue Crew Player Summary: role (Captain/Couple/—), game counts, ordered partners

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/ATH_Open_Sheets_Template.xlsx
+++ b/backend/ATH_Open_Sheets_Template.xlsx
@@ -10,6 +10,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Players" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Schedule" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How To Use" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Full Schedule" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSB Pairings Matrix" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HSB Player Summary" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blue Crew Matrix" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blue Crew Player Summary" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +40,60 @@
       <b val="1"/>
     </font>
     <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B4F00"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="005E2CA5"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -78,6 +135,31 @@
         <fgColor rgb="002d7d4f"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF176"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E0E0E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C8E6C9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -105,7 +187,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -131,6 +213,129 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2651,4 +2856,3187 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ATH Open — Full Tournament Schedule  (Hill Street Blues  vs  Blue Crew / JPL Team)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Round</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Time</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Court</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Hill Street Blues</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr"/>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>Blue Crew (JPL)</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr"/>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="13" t="n"/>
+      <c r="B3" s="13" t="n"/>
+      <c r="C3" s="13" t="n"/>
+      <c r="D3" s="13" t="n"/>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Player 1</t>
+        </is>
+      </c>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Player 2</t>
+        </is>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>Player 1</t>
+        </is>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>Player 2</t>
+        </is>
+      </c>
+      <c r="I3" s="13" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>Jeff E</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>8:30 AM</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Dro</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>8:50 AM</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
+        <is>
+          <t>Mich</t>
+        </is>
+      </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>Wilfred</t>
+        </is>
+      </c>
+      <c r="G6" s="14" t="inlineStr">
+        <is>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="H6" s="14" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="I6" s="14" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>8:50 AM</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
+        <is>
+          <t>Jeff W</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Yu Fon</t>
+        </is>
+      </c>
+      <c r="G7" s="14" t="inlineStr">
+        <is>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="H7" s="14" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="I7" s="14" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>9:15 AM</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Jeff W</t>
+        </is>
+      </c>
+      <c r="G8" s="14" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="H8" s="14" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="I8" s="14" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>9:15 AM</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
+          <t>Dro</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>Johnny</t>
+        </is>
+      </c>
+      <c r="G9" s="14" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="H9" s="14" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>9:40 AM</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D10" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E10" s="15" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>Suzan</t>
+        </is>
+      </c>
+      <c r="G10" s="15" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="I10" s="15" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="15" t="inlineStr">
+        <is>
+          <t>9:40 AM</t>
+        </is>
+      </c>
+      <c r="C11" s="15" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Jeff E</t>
+        </is>
+      </c>
+      <c r="F11" s="15" t="inlineStr">
+        <is>
+          <t>Rachel</t>
+        </is>
+      </c>
+      <c r="G11" s="15" t="inlineStr">
+        <is>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="I11" s="15" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="15" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>10:10 AM</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>Jeff E</t>
+        </is>
+      </c>
+      <c r="F12" s="15" t="inlineStr">
+        <is>
+          <t>Molly</t>
+        </is>
+      </c>
+      <c r="G12" s="15" t="inlineStr">
+        <is>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="I12" s="15" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>10:10 AM</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E13" s="14" t="inlineStr">
+        <is>
+          <t>Johnny</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
+          <t>Wilfred</t>
+        </is>
+      </c>
+      <c r="G13" s="14" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="H13" s="14" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Yu Fon</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="inlineStr">
+        <is>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="H14" s="14" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="I14" s="14" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="14" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="14" t="inlineStr">
+        <is>
+          <t>10:30 AM</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="F15" s="14" t="inlineStr">
+        <is>
+          <t>Mich</t>
+        </is>
+      </c>
+      <c r="G15" s="14" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="H15" s="14" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="I15" s="14" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>Johnny</t>
+        </is>
+      </c>
+      <c r="F16" s="15" t="inlineStr">
+        <is>
+          <t>Rachel</t>
+        </is>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="I16" s="15" t="inlineStr">
+        <is>
+          <t>Captain's game ★</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>11:00 AM</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>Mich</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>Molly</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D18" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="inlineStr">
+        <is>
+          <t>Jeff W</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="inlineStr">
+        <is>
+          <t>Dro</t>
+        </is>
+      </c>
+      <c r="G18" s="14" t="inlineStr">
+        <is>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="H18" s="14" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="I18" s="14" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="14" t="n">
+        <v>8</v>
+      </c>
+      <c r="B19" s="14" t="inlineStr">
+        <is>
+          <t>11:30 AM</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="inlineStr">
+        <is>
+          <t>Men's Doubles</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="inlineStr">
+        <is>
+          <t>Yu Fon</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="inlineStr">
+        <is>
+          <t>Jeff E</t>
+        </is>
+      </c>
+      <c r="G19" s="14" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="H19" s="14" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="I19" s="14" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>S (South)</t>
+        </is>
+      </c>
+      <c r="D20" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E20" s="15" t="inlineStr">
+        <is>
+          <t>Wilfred</t>
+        </is>
+      </c>
+      <c r="F20" s="15" t="inlineStr">
+        <is>
+          <t>Rachel</t>
+        </is>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="I20" s="15" t="n"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="15" t="n">
+        <v>9</v>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>N (North)</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
+          <t>Mix Doubles ★</t>
+        </is>
+      </c>
+      <c r="E21" s="15" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="F21" s="15" t="inlineStr">
+        <is>
+          <t>Molly</t>
+        </is>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="I21" s="15" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Hill Street Blues — Player Pairings Matrix   (X = Men's Doubles  |  M★ = Mixed Doubles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Captain: Suzan  ·  No fixed couples  ·  3 women × 1–3 mixed games  ·  9 men × 3–4 games each</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>Pierre
+(M)</t>
+        </is>
+      </c>
+      <c r="D4" s="18" t="inlineStr">
+        <is>
+          <t>Jeff E
+(M)</t>
+        </is>
+      </c>
+      <c r="E4" s="18" t="inlineStr">
+        <is>
+          <t>Dro
+(M)</t>
+        </is>
+      </c>
+      <c r="F4" s="18" t="inlineStr">
+        <is>
+          <t>Steve
+(M)</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Mich
+(M)</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Wilfred
+(M)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Jeff W
+(M)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Yu Fon
+(M)</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Johnny
+(M)</t>
+        </is>
+      </c>
+      <c r="L4" s="19" t="inlineStr">
+        <is>
+          <t>Suzan
+(F★) ©</t>
+        </is>
+      </c>
+      <c r="M4" s="19" t="inlineStr">
+        <is>
+          <t>Rachel
+(F★)</t>
+        </is>
+      </c>
+      <c r="N4" s="19" t="inlineStr">
+        <is>
+          <t>Molly
+(F★)</t>
+        </is>
+      </c>
+      <c r="O4" s="13" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>Mix★</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Pierre (M)</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-S</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-N</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="24" t="n"/>
+      <c r="K5" s="24" t="n"/>
+      <c r="L5" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-S</t>
+        </is>
+      </c>
+      <c r="M5" s="24" t="n"/>
+      <c r="N5" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R9-N</t>
+        </is>
+      </c>
+      <c r="O5" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="P5" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="20" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Jeff E (M)</t>
+        </is>
+      </c>
+      <c r="C6" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-S</t>
+        </is>
+      </c>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-N</t>
+        </is>
+      </c>
+      <c r="K6" s="24" t="n"/>
+      <c r="L6" s="24" t="n"/>
+      <c r="M6" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-N</t>
+        </is>
+      </c>
+      <c r="N6" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R5-S</t>
+        </is>
+      </c>
+      <c r="O6" s="26" t="n">
+        <v>4</v>
+      </c>
+      <c r="P6" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Dro (M)</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-N</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="n"/>
+      <c r="H7" s="24" t="n"/>
+      <c r="I7" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-S</t>
+        </is>
+      </c>
+      <c r="J7" s="24" t="n"/>
+      <c r="K7" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-N</t>
+        </is>
+      </c>
+      <c r="L7" s="24" t="n"/>
+      <c r="M7" s="24" t="n"/>
+      <c r="N7" s="24" t="n"/>
+      <c r="O7" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P7" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Steve (M)</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-N</t>
+        </is>
+      </c>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-S</t>
+        </is>
+      </c>
+      <c r="J8" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-S</t>
+        </is>
+      </c>
+      <c r="K8" s="24" t="n"/>
+      <c r="L8" s="24" t="n"/>
+      <c r="M8" s="24" t="n"/>
+      <c r="N8" s="24" t="n"/>
+      <c r="O8" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P8" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Mich (M)</t>
+        </is>
+      </c>
+      <c r="C9" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-N</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-S</t>
+        </is>
+      </c>
+      <c r="I9" s="24" t="n"/>
+      <c r="J9" s="24" t="n"/>
+      <c r="K9" s="24" t="n"/>
+      <c r="L9" s="24" t="n"/>
+      <c r="M9" s="24" t="n"/>
+      <c r="N9" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R7-N</t>
+        </is>
+      </c>
+      <c r="O9" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P9" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Wilfred (M)</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="24" t="n"/>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-S</t>
+        </is>
+      </c>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="24" t="n"/>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>X
+R5-N</t>
+        </is>
+      </c>
+      <c r="L10" s="24" t="n"/>
+      <c r="M10" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R9-S</t>
+        </is>
+      </c>
+      <c r="N10" s="24" t="n"/>
+      <c r="O10" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P10" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Jeff W (M)</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-S</t>
+        </is>
+      </c>
+      <c r="F11" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-S</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="n"/>
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-N</t>
+        </is>
+      </c>
+      <c r="K11" s="24" t="n"/>
+      <c r="L11" s="24" t="n"/>
+      <c r="M11" s="24" t="n"/>
+      <c r="N11" s="24" t="n"/>
+      <c r="O11" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P11" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Yu Fon (M)</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-N</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-S</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="n"/>
+      <c r="H12" s="24" t="n"/>
+      <c r="I12" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-N</t>
+        </is>
+      </c>
+      <c r="J12" s="22" t="n"/>
+      <c r="K12" s="24" t="n"/>
+      <c r="L12" s="24" t="n"/>
+      <c r="M12" s="24" t="n"/>
+      <c r="N12" s="24" t="n"/>
+      <c r="O12" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P12" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Johnny (M)</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-N</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
+      <c r="H13" s="23" t="inlineStr">
+        <is>
+          <t>X
+R5-N</t>
+        </is>
+      </c>
+      <c r="I13" s="24" t="n"/>
+      <c r="J13" s="24" t="n"/>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="24" t="n"/>
+      <c r="M13" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R7-S</t>
+        </is>
+      </c>
+      <c r="N13" s="24" t="n"/>
+      <c r="O13" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="P13" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="28" t="inlineStr">
+        <is>
+          <t>Suzan (F) ©</t>
+        </is>
+      </c>
+      <c r="C14" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-S</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="24" t="n"/>
+      <c r="G14" s="24" t="n"/>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="24" t="n"/>
+      <c r="J14" s="24" t="n"/>
+      <c r="K14" s="24" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="24" t="n"/>
+      <c r="N14" s="24" t="n"/>
+      <c r="O14" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="P14" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="27" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t>Rachel (F)</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-N</t>
+        </is>
+      </c>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="24" t="n"/>
+      <c r="G15" s="24" t="n"/>
+      <c r="H15" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R9-S</t>
+        </is>
+      </c>
+      <c r="I15" s="24" t="n"/>
+      <c r="J15" s="24" t="n"/>
+      <c r="K15" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R7-S</t>
+        </is>
+      </c>
+      <c r="L15" s="24" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="24" t="n"/>
+      <c r="O15" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="P15" s="15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="27" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="28" t="inlineStr">
+        <is>
+          <t>Molly (F)</t>
+        </is>
+      </c>
+      <c r="C16" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R9-N</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R5-S</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="24" t="n"/>
+      <c r="G16" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R7-N</t>
+        </is>
+      </c>
+      <c r="H16" s="24" t="n"/>
+      <c r="I16" s="24" t="n"/>
+      <c r="J16" s="24" t="n"/>
+      <c r="K16" s="24" t="n"/>
+      <c r="L16" s="24" t="n"/>
+      <c r="M16" s="24" t="n"/>
+      <c r="N16" s="22" t="n"/>
+      <c r="O16" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="P16" s="15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Games</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Men's Dbl</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Mixed★</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Games in order (round-court)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="31" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D2" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E2" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F2" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H2" s="33" t="inlineStr">
+        <is>
+          <t>R1-S w/Jeff E,  R4-S★ w/Suzan,  R6-N w/Mich,  R9-N★ w/Molly</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="31" t="inlineStr">
+        <is>
+          <t>Jeff E</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E3" s="32" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="33" t="inlineStr">
+        <is>
+          <t>R1-S w/Pierre,  R4-N★ w/Rachel,  R5-S★ w/Molly,  R8-N w/Yu Fon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Dro</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E4" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="33" t="inlineStr">
+        <is>
+          <t>R1-N w/Steve,  R3-N w/Johnny,  R8-S w/Jeff W</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="31" t="inlineStr">
+        <is>
+          <t>Steve</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="33" t="inlineStr">
+        <is>
+          <t>R1-N w/Dro,  R3-S w/Jeff W,  R6-S w/Yu Fon</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Mich</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>R2-S w/Wilfred,  R6-N w/Pierre,  R7-N★ w/Molly</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Wilfred</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>R2-S w/Mich,  R5-N w/Johnny,  R9-S★ w/Rachel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Jeff W</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t>R2-N w/Yu Fon,  R3-S w/Steve,  R8-S w/Dro</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Yu Fon</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>R2-N w/Jeff W,  R6-S w/Steve,  R8-N w/Jeff E</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Johnny</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G10" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>R3-N w/Dro,  R5-N w/Wilfred,  R7-S★ w/Rachel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="34" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="35" t="inlineStr">
+        <is>
+          <t>Suzan</t>
+        </is>
+      </c>
+      <c r="C11" s="34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D11" s="34" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="37" t="inlineStr">
+        <is>
+          <t>R4-S★ w/Pierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="34" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Rachel</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="37" t="inlineStr">
+        <is>
+          <t>R4-N★ w/Jeff E,  R7-S★ w/Johnny,  R9-S★ w/Wilfred</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="34" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="35" t="inlineStr">
+        <is>
+          <t>Molly</t>
+        </is>
+      </c>
+      <c r="C13" s="34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="H13" s="37" t="inlineStr">
+        <is>
+          <t>R5-S★ w/Jeff E,  R7-N★ w/Mich,  R9-N★ w/Pierre</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Blue Crew (JPL Team) — Pairings Matrix   (X = Men's Doubles  |  M★ = Mixed Doubles  |  C★ = Captain's game)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="17" t="inlineStr">
+        <is>
+          <t>Captain: Cora (1 game w/ Jay)  ·  Couples: Trevor↔Alexis, Marv↔Carmela, Pierre↔Ivy  ·  No back-to-back games</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="6" customHeight="1"/>
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C4" s="38" t="inlineStr">
+        <is>
+          <t>Cora
+(C★)</t>
+        </is>
+      </c>
+      <c r="D4" s="19" t="inlineStr">
+        <is>
+          <t>Alexis
+(F)</t>
+        </is>
+      </c>
+      <c r="E4" s="19" t="inlineStr">
+        <is>
+          <t>Carmela
+(F)</t>
+        </is>
+      </c>
+      <c r="F4" s="19" t="inlineStr">
+        <is>
+          <t>Ivy
+(F)</t>
+        </is>
+      </c>
+      <c r="G4" s="18" t="inlineStr">
+        <is>
+          <t>Jay
+(M)</t>
+        </is>
+      </c>
+      <c r="H4" s="18" t="inlineStr">
+        <is>
+          <t>Marv
+(M)</t>
+        </is>
+      </c>
+      <c r="I4" s="18" t="inlineStr">
+        <is>
+          <t>Arman
+(M)</t>
+        </is>
+      </c>
+      <c r="J4" s="18" t="inlineStr">
+        <is>
+          <t>Jon
+(M)</t>
+        </is>
+      </c>
+      <c r="K4" s="18" t="inlineStr">
+        <is>
+          <t>Trevor
+(M)</t>
+        </is>
+      </c>
+      <c r="L4" s="18" t="inlineStr">
+        <is>
+          <t>Richard
+(M)</t>
+        </is>
+      </c>
+      <c r="M4" s="18" t="inlineStr">
+        <is>
+          <t>Rhon
+(M)</t>
+        </is>
+      </c>
+      <c r="N4" s="18" t="inlineStr">
+        <is>
+          <t>Joe
+(M)</t>
+        </is>
+      </c>
+      <c r="O4" s="18" t="inlineStr">
+        <is>
+          <t>Pierre
+(M)</t>
+        </is>
+      </c>
+      <c r="P4" s="13" t="inlineStr">
+        <is>
+          <t>Games</t>
+        </is>
+      </c>
+      <c r="Q4" s="13" t="inlineStr">
+        <is>
+          <t>Mix★</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Cora (C★) Captain</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="41" t="inlineStr">
+        <is>
+          <t>C★
+R7-S</t>
+        </is>
+      </c>
+      <c r="H5" s="24" t="n"/>
+      <c r="I5" s="24" t="n"/>
+      <c r="J5" s="24" t="n"/>
+      <c r="K5" s="24" t="n"/>
+      <c r="L5" s="24" t="n"/>
+      <c r="M5" s="24" t="n"/>
+      <c r="N5" s="24" t="n"/>
+      <c r="O5" s="24" t="n"/>
+      <c r="P5" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="27" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Alexis (F)</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="24" t="n"/>
+      <c r="F6" s="24" t="n"/>
+      <c r="G6" s="24" t="n"/>
+      <c r="H6" s="24" t="n"/>
+      <c r="I6" s="24" t="n"/>
+      <c r="J6" s="24" t="n"/>
+      <c r="K6" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R5-S,R9-S</t>
+        </is>
+      </c>
+      <c r="L6" s="24" t="n"/>
+      <c r="M6" s="24" t="n"/>
+      <c r="N6" s="24" t="n"/>
+      <c r="O6" s="24" t="n"/>
+      <c r="P6" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Carmela (F)</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="n"/>
+      <c r="D7" s="24" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="24" t="n"/>
+      <c r="G7" s="24" t="n"/>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-N,R9-N</t>
+        </is>
+      </c>
+      <c r="I7" s="24" t="n"/>
+      <c r="J7" s="24" t="n"/>
+      <c r="K7" s="24" t="n"/>
+      <c r="L7" s="24" t="n"/>
+      <c r="M7" s="24" t="n"/>
+      <c r="N7" s="24" t="n"/>
+      <c r="O7" s="24" t="n"/>
+      <c r="P7" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Ivy (F)</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="n"/>
+      <c r="D8" s="24" t="n"/>
+      <c r="E8" s="24" t="n"/>
+      <c r="F8" s="22" t="n"/>
+      <c r="G8" s="24" t="n"/>
+      <c r="H8" s="24" t="n"/>
+      <c r="I8" s="24" t="n"/>
+      <c r="J8" s="24" t="n"/>
+      <c r="K8" s="24" t="n"/>
+      <c r="L8" s="24" t="n"/>
+      <c r="M8" s="24" t="n"/>
+      <c r="N8" s="24" t="n"/>
+      <c r="O8" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-S,R7-N</t>
+        </is>
+      </c>
+      <c r="P8" s="29" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q8" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Jay (M)</t>
+        </is>
+      </c>
+      <c r="C9" s="41" t="inlineStr">
+        <is>
+          <t>C★
+R7-S</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="22" t="n"/>
+      <c r="H9" s="24" t="n"/>
+      <c r="I9" s="24" t="n"/>
+      <c r="J9" s="24" t="n"/>
+      <c r="K9" s="24" t="n"/>
+      <c r="L9" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-N</t>
+        </is>
+      </c>
+      <c r="M9" s="23" t="inlineStr">
+        <is>
+          <t>X
+R5-N</t>
+        </is>
+      </c>
+      <c r="N9" s="24" t="n"/>
+      <c r="O9" s="24" t="n"/>
+      <c r="P9" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q9" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Marv (M)</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-N,R9-N</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="n"/>
+      <c r="G10" s="24" t="n"/>
+      <c r="H10" s="22" t="n"/>
+      <c r="I10" s="24" t="n"/>
+      <c r="J10" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-N</t>
+        </is>
+      </c>
+      <c r="K10" s="24" t="n"/>
+      <c r="L10" s="24" t="n"/>
+      <c r="M10" s="24" t="n"/>
+      <c r="N10" s="24" t="n"/>
+      <c r="O10" s="24" t="n"/>
+      <c r="P10" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q10" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="20" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Arman (M)</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
+      <c r="H11" s="24" t="n"/>
+      <c r="I11" s="22" t="n"/>
+      <c r="J11" s="24" t="n"/>
+      <c r="K11" s="24" t="n"/>
+      <c r="L11" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-S</t>
+        </is>
+      </c>
+      <c r="M11" s="24" t="n"/>
+      <c r="N11" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-S</t>
+        </is>
+      </c>
+      <c r="O11" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-S</t>
+        </is>
+      </c>
+      <c r="P11" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q11" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="20" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Jon (M)</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="24" t="n"/>
+      <c r="F12" s="24" t="n"/>
+      <c r="G12" s="24" t="n"/>
+      <c r="H12" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-N</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="n"/>
+      <c r="J12" s="22" t="n"/>
+      <c r="K12" s="24" t="n"/>
+      <c r="L12" s="24" t="n"/>
+      <c r="M12" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-N</t>
+        </is>
+      </c>
+      <c r="N12" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-N</t>
+        </is>
+      </c>
+      <c r="O12" s="24" t="n"/>
+      <c r="P12" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q12" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="20" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Trevor (M)</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R5-S,R9-S</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
+      <c r="H13" s="24" t="n"/>
+      <c r="I13" s="24" t="n"/>
+      <c r="J13" s="24" t="n"/>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="24" t="n"/>
+      <c r="M13" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-S</t>
+        </is>
+      </c>
+      <c r="N13" s="24" t="n"/>
+      <c r="O13" s="24" t="n"/>
+      <c r="P13" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1">
+      <c r="A14" s="20" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Richard (M)</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="24" t="n"/>
+      <c r="G14" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-N</t>
+        </is>
+      </c>
+      <c r="H14" s="24" t="n"/>
+      <c r="I14" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-S</t>
+        </is>
+      </c>
+      <c r="J14" s="24" t="n"/>
+      <c r="K14" s="24" t="n"/>
+      <c r="L14" s="22" t="n"/>
+      <c r="M14" s="24" t="n"/>
+      <c r="N14" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-N</t>
+        </is>
+      </c>
+      <c r="O14" s="24" t="n"/>
+      <c r="P14" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="20" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Rhon (M)</t>
+        </is>
+      </c>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="24" t="n"/>
+      <c r="F15" s="24" t="n"/>
+      <c r="G15" s="23" t="inlineStr">
+        <is>
+          <t>X
+R5-N</t>
+        </is>
+      </c>
+      <c r="H15" s="24" t="n"/>
+      <c r="I15" s="24" t="n"/>
+      <c r="J15" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-N</t>
+        </is>
+      </c>
+      <c r="K15" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-S</t>
+        </is>
+      </c>
+      <c r="L15" s="24" t="n"/>
+      <c r="M15" s="22" t="n"/>
+      <c r="N15" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-S</t>
+        </is>
+      </c>
+      <c r="O15" s="24" t="n"/>
+      <c r="P15" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="20" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Joe (M)</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="n"/>
+      <c r="D16" s="24" t="n"/>
+      <c r="E16" s="24" t="n"/>
+      <c r="F16" s="24" t="n"/>
+      <c r="G16" s="24" t="n"/>
+      <c r="H16" s="24" t="n"/>
+      <c r="I16" s="23" t="inlineStr">
+        <is>
+          <t>X
+R8-S</t>
+        </is>
+      </c>
+      <c r="J16" s="23" t="inlineStr">
+        <is>
+          <t>X
+R6-N</t>
+        </is>
+      </c>
+      <c r="K16" s="24" t="n"/>
+      <c r="L16" s="23" t="inlineStr">
+        <is>
+          <t>X
+R1-N</t>
+        </is>
+      </c>
+      <c r="M16" s="23" t="inlineStr">
+        <is>
+          <t>X
+R3-S</t>
+        </is>
+      </c>
+      <c r="N16" s="22" t="n"/>
+      <c r="O16" s="24" t="n"/>
+      <c r="P16" s="43" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q16" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="20" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Pierre (M)</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="25" t="inlineStr">
+        <is>
+          <t>M★
+R4-S,R7-N</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="n"/>
+      <c r="H17" s="24" t="n"/>
+      <c r="I17" s="23" t="inlineStr">
+        <is>
+          <t>X
+R2-S</t>
+        </is>
+      </c>
+      <c r="J17" s="24" t="n"/>
+      <c r="K17" s="24" t="n"/>
+      <c r="L17" s="24" t="n"/>
+      <c r="M17" s="24" t="n"/>
+      <c r="N17" s="24" t="n"/>
+      <c r="O17" s="22" t="n"/>
+      <c r="P17" s="26" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q17" s="15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Total Games</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Men's Dbl</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Mixed★</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Games in order (round-court)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="45" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="C2" s="44" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D2" s="44" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="E2" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="47" t="inlineStr">
+        <is>
+          <t>R7-S★ w/Jay</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="C3" s="34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D3" s="34" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E3" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="37" t="inlineStr">
+        <is>
+          <t>R5-S★ w/Trevor,  R9-S★ w/Trevor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="34" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="37" t="inlineStr">
+        <is>
+          <t>R4-N★ w/Marv,  R9-N★ w/Marv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="C5" s="34" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D5" s="34" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="37" t="inlineStr">
+        <is>
+          <t>R4-S★ w/Pierre,  R7-N★ w/Pierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="30" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="31" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D6" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="33" t="inlineStr">
+        <is>
+          <t>R3-N w/Richard,  R5-N w/Rhon,  R7-S★ w/Cora</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="31" t="inlineStr">
+        <is>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="33" t="inlineStr">
+        <is>
+          <t>R2-N w/Jon,  R4-N★ w/Carmela,  R9-N★ w/Carmela</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="30" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="31" t="inlineStr">
+        <is>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="33" t="inlineStr">
+        <is>
+          <t>R2-S w/Pierre,  R6-S w/Richard,  R8-S w/Joe</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="31" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>R2-N w/Marv,  R6-N w/Joe,  R8-N w/Rhon</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="30" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="31" t="inlineStr">
+        <is>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="33" t="inlineStr">
+        <is>
+          <t>R1-S w/Rhon,  R5-S★ w/Alexis,  R9-S★ w/Alexis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="30" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="31" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="33" t="inlineStr">
+        <is>
+          <t>R1-N w/Joe,  R3-N w/Jay,  R6-S w/Arman</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="48" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="49" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="C12" s="48" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D12" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="51" t="inlineStr">
+        <is>
+          <t>R1-S w/Trevor,  R3-S w/Joe,  R5-N w/Jay,  R8-N w/Jon</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="C13" s="48" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D13" s="48" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="50" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="48" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="51" t="inlineStr">
+        <is>
+          <t>R1-N w/Richard,  R3-S w/Rhon,  R6-N w/Jon,  R8-S w/Arman</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="30" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="31" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>R2-S w/Arman,  R4-S★ w/Ivy,  R7-N★ w/Ivy</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Disambiguate Blue Crew Pierre as "Pierre Y"
Both teams have a Pierre — Blue Crew's is Pierre Y (b12), HSB's stays as Pierre (a4).
Updated mockData.js, generate_template.py, and regenerated the xlsx.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/ATH_Open_Sheets_Template.xlsx
+++ b/backend/ATH_Open_Sheets_Template.xlsx
@@ -1605,7 +1605,11 @@
           <t>Pierre</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
           <t>B</t>
@@ -3069,7 +3073,7 @@
       </c>
       <c r="H6" s="14" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Pierre Y</t>
         </is>
       </c>
       <c r="I6" s="14" t="n"/>
@@ -3228,7 +3232,7 @@
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Pierre Y</t>
         </is>
       </c>
       <c r="H10" s="15" t="inlineStr">
@@ -3519,7 +3523,7 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Pierre Y</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -4972,7 +4976,7 @@
       </c>
       <c r="O4" s="18" t="inlineStr">
         <is>
-          <t>Pierre
+          <t>Pierre Y
 (M)</t>
         </is>
       </c>
@@ -5491,7 +5495,7 @@
       </c>
       <c r="B17" s="21" t="inlineStr">
         <is>
-          <t>Pierre (M)</t>
+          <t>Pierre Y (M)</t>
         </is>
       </c>
       <c r="C17" s="24" t="n"/>
@@ -5726,7 +5730,7 @@
       </c>
       <c r="H5" s="37" t="inlineStr">
         <is>
-          <t>R4-S★ w/Pierre,  R7-N★ w/Pierre</t>
+          <t>R4-S★ w/Pierre Y,  R7-N★ w/Pierre Y</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5832,7 @@
       </c>
       <c r="H8" s="33" t="inlineStr">
         <is>
-          <t>R2-S w/Pierre,  R6-S w/Richard,  R8-S w/Joe</t>
+          <t>R2-S w/Pierre Y,  R6-S w/Richard,  R8-S w/Joe</t>
         </is>
       </c>
     </row>
@@ -6008,7 +6012,7 @@
       </c>
       <c r="B14" s="31" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Pierre Y</t>
         </is>
       </c>
       <c r="C14" s="30" t="inlineStr">

</xml_diff>